<commit_message>
Filter matching COMET full-sequence distance exports
</commit_message>
<xml_diff>
--- a/HCVData/subtyping-comparison-all-ras/11-report-subtype-agreement/NS5A_CometFullSeqSubtype_4R_Subtyping_Distances.xlsx
+++ b/HCVData/subtyping-comparison-all-ras/11-report-subtype-agreement/NS5A_CometFullSeqSubtype_4R_Subtyping_Distances.xlsx
@@ -9,13 +9,6 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Genotype" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Subtype_1" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Subtype_2" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Subtype_3" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Subtype_4" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Subtype_5" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Subtype_6" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Subtype_7" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Subtype_8" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2754,924 +2747,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Accession</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>CometFullSeqSubtype</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>ClosestSubtypeAlignedNT</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>AssignedGenotype</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Subtype2aDistance</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Subtype2aDistance</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Subtype2bDistance</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Subtype2bDistance</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Subtype2cDistance</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Subtype2dDistance</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Subtype2eDistance</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Subtype2fDistance</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Subtype2fDistance</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>Subtype2iDistance</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>Subtype2jDistance</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>Subtype2jDistance</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>Subtype2kDistance</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>Subtype2lDistance</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>Subtype2lDistance</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>Subtype2mDistance</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>Subtype2mDistance</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>Subtype2qDistance</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>Subtype2qDistance</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>Subtype2rDistance</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>Subtype2tDistance</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>Subtype2uDistance</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>Subtype2vDistance</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>FirstChoiceSubtype</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>FirstChoiceDistance</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>SecondChoiceSubtype</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>SecondChoiceDistance</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Accession</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>CometFullSeqSubtype</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>ClosestSubtypeAlignedNT</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>AssignedGenotype</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Subtype3aDistance</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Subtype3bDistance</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Subtype3dDistance</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Subtype3eDistance</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Subtype3gDistance</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Subtype3gDistance</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Subtype3hDistance</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Subtype3iDistance</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Subtype3iDistance</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>Subtype3kDistance</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>Subtype3kDistance</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>FirstChoiceSubtype</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>FirstChoiceDistance</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>SecondChoiceSubtype</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>SecondChoiceDistance</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Accession</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>CometFullSeqSubtype</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>ClosestSubtypeAlignedNT</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>AssignedGenotype</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Subtype4aDistance</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Subtype4bDistance</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Subtype4cDistance</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Subtype4dDistance</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Subtype4dDistance</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Subtype4fDistance</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Subtype4fDistance</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Subtype4gDistance</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Subtype4kDistance</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>Subtype4kDistance</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>Subtype4lDistance</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>Subtype4mDistance</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>Subtype4nDistance</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>Subtype4oDistance</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>Subtype4pDistance</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>Subtype4qDistance</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>Subtype4rDistance</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>Subtype4sDistance</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>Subtype4tDistance</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>Subtype4vDistance</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>Subtype4vDistance</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>Subtype4wDistance</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>Subtype4wDistance</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>FirstChoiceSubtype</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>FirstChoiceDistance</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>SecondChoiceSubtype</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>SecondChoiceDistance</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Accession</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>CometFullSeqSubtype</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>ClosestSubtypeAlignedNT</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>AssignedGenotype</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Subtype5aDistance</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Subtype5bDistance</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>FirstChoiceSubtype</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>FirstChoiceDistance</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>SecondChoiceSubtype</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>SecondChoiceDistance</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Accession</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>CometFullSeqSubtype</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>ClosestSubtypeAlignedNT</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>AssignedGenotype</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Subtype6aDistance</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Subtype6aDistance</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Subtype6bDistance</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Subtype6cDistance</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Subtype6dDistance</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Subtype6eDistance</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Subtype6fDistance</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Subtype6gDistance</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Subtype6hDistance</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>Subtype6iDistance</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>Subtype6jDistance</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>Subtype6kDistance</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>Subtype6lDistance</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>Subtype6mDistance</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>Subtype6nDistance</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>Subtype6nDistance</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>Subtype6oDistance</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>Subtype6pDistance</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>Subtype6qDistance</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>Subtype6rDistance</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>Subtype6sDistance</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>Subtype6tDistance</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>Subtype6tDistance</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>Subtype6uDistance</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>Subtype6vDistance</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>Subtype6vDistance</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>Subtype6wDistance</t>
-        </is>
-      </c>
-      <c r="AF1" t="inlineStr">
-        <is>
-          <t>Subtype6wDistance</t>
-        </is>
-      </c>
-      <c r="AG1" t="inlineStr">
-        <is>
-          <t>Subtype6xaDistance</t>
-        </is>
-      </c>
-      <c r="AH1" t="inlineStr">
-        <is>
-          <t>Subtype6xaDistance</t>
-        </is>
-      </c>
-      <c r="AI1" t="inlineStr">
-        <is>
-          <t>Subtype6xbDistance</t>
-        </is>
-      </c>
-      <c r="AJ1" t="inlineStr">
-        <is>
-          <t>Subtype6xbDistance</t>
-        </is>
-      </c>
-      <c r="AK1" t="inlineStr">
-        <is>
-          <t>Subtype6xcDistance</t>
-        </is>
-      </c>
-      <c r="AL1" t="inlineStr">
-        <is>
-          <t>Subtype6xdDistance</t>
-        </is>
-      </c>
-      <c r="AM1" t="inlineStr">
-        <is>
-          <t>Subtype6xdDistance</t>
-        </is>
-      </c>
-      <c r="AN1" t="inlineStr">
-        <is>
-          <t>Subtype6xeDistance</t>
-        </is>
-      </c>
-      <c r="AO1" t="inlineStr">
-        <is>
-          <t>Subtype6xeDistance</t>
-        </is>
-      </c>
-      <c r="AP1" t="inlineStr">
-        <is>
-          <t>Subtype6xfDistance</t>
-        </is>
-      </c>
-      <c r="AQ1" t="inlineStr">
-        <is>
-          <t>Subtype6xfDistance</t>
-        </is>
-      </c>
-      <c r="AR1" t="inlineStr">
-        <is>
-          <t>Subtype6xgDistance</t>
-        </is>
-      </c>
-      <c r="AS1" t="inlineStr">
-        <is>
-          <t>Subtype6xgDistance</t>
-        </is>
-      </c>
-      <c r="AT1" t="inlineStr">
-        <is>
-          <t>Subtype6xhDistance</t>
-        </is>
-      </c>
-      <c r="AU1" t="inlineStr">
-        <is>
-          <t>Subtype6xiDistance</t>
-        </is>
-      </c>
-      <c r="AV1" t="inlineStr">
-        <is>
-          <t>Subtype6xiDistance</t>
-        </is>
-      </c>
-      <c r="AW1" t="inlineStr">
-        <is>
-          <t>Subtype6xjDistance</t>
-        </is>
-      </c>
-      <c r="AX1" t="inlineStr">
-        <is>
-          <t>FirstChoiceSubtype</t>
-        </is>
-      </c>
-      <c r="AY1" t="inlineStr">
-        <is>
-          <t>FirstChoiceDistance</t>
-        </is>
-      </c>
-      <c r="AZ1" t="inlineStr">
-        <is>
-          <t>SecondChoiceSubtype</t>
-        </is>
-      </c>
-      <c r="BA1" t="inlineStr">
-        <is>
-          <t>SecondChoiceDistance</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Accession</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>CometFullSeqSubtype</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>ClosestSubtypeAlignedNT</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>AssignedGenotype</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Subtype7aDistance</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Subtype7bDistance</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>FirstChoiceSubtype</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>FirstChoiceDistance</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>SecondChoiceSubtype</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>SecondChoiceDistance</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Accession</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>CometFullSeqSubtype</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>ClosestSubtypeAlignedNT</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>AssignedGenotype</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Subtype8aDistance</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>FirstChoiceSubtype</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>FirstChoiceDistance</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>SecondChoiceSubtype</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>SecondChoiceDistance</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>